<commit_message>
Añadido el word con la gestion de riesgos
</commit_message>
<xml_diff>
--- a/_ANALISIS DE RIESGOS.xlsx
+++ b/_ANALISIS DE RIESGOS.xlsx
@@ -1,20 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Documents\Universidad\SEGUNDO\IS1\Proyecto-IS1\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1F22416-6BDA-44B7-8828-8F9AD7764DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="612" yWindow="588" windowWidth="21852" windowHeight="8676"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="67">
   <si>
     <t>RIESGO</t>
   </si>
@@ -212,13 +231,16 @@
   </si>
   <si>
     <t>Improbable</t>
+  </si>
+  <si>
+    <t>NOTA: Los riesgos que se analizarán en profundidad son los resaltados en amarillo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -271,8 +293,15 @@
       <color rgb="FF000000"/>
       <name val="&quot;Aptos Narrow&quot;"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -323,12 +352,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -384,6 +407,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2"/>
+        <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
@@ -452,13 +487,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+  <cellXfs count="56">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -468,55 +503,59 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -527,12 +566,11 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -732,7 +770,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -749,8 +787,10 @@
     <col min="11" max="11" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:11">
-      <c r="C3" s="1"/>
+    <row r="3" spans="1:11" ht="13.2">
+      <c r="C3" s="55" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="5" spans="1:11" ht="13.8">
       <c r="C5" s="9" t="s">
@@ -794,8 +834,8 @@
       <c r="G6" s="4">
         <v>4</v>
       </c>
-      <c r="H6" s="52">
-        <f t="shared" ref="H6:H39" si="0">E6*G6</f>
+      <c r="H6" s="51">
+        <f t="shared" ref="H6:H38" si="0">E6*G6</f>
         <v>12</v>
       </c>
       <c r="I6" s="2"/>
@@ -810,7 +850,7 @@
       <c r="B7" s="6">
         <v>2</v>
       </c>
-      <c r="C7" s="47" t="s">
+      <c r="C7" s="46" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="16" t="s">
@@ -825,7 +865,7 @@
       <c r="G7" s="5">
         <v>2</v>
       </c>
-      <c r="H7" s="53">
+      <c r="H7" s="52">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
@@ -841,7 +881,7 @@
       <c r="B8" s="6">
         <v>3</v>
       </c>
-      <c r="C8" s="47" t="s">
+      <c r="C8" s="46" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="27" t="s">
@@ -856,7 +896,7 @@
       <c r="G8" s="4">
         <v>3</v>
       </c>
-      <c r="H8" s="53">
+      <c r="H8" s="52">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
@@ -887,7 +927,7 @@
       <c r="G9" s="5">
         <v>3</v>
       </c>
-      <c r="H9" s="52">
+      <c r="H9" s="51">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
@@ -918,7 +958,7 @@
       <c r="G10" s="4">
         <v>5</v>
       </c>
-      <c r="H10" s="52">
+      <c r="H10" s="51">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
@@ -949,7 +989,7 @@
       <c r="G11" s="5">
         <v>3</v>
       </c>
-      <c r="H11" s="52">
+      <c r="H11" s="51">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
@@ -965,7 +1005,7 @@
       <c r="B12" s="6">
         <v>7</v>
       </c>
-      <c r="C12" s="48" t="s">
+      <c r="C12" s="47" t="s">
         <v>19</v>
       </c>
       <c r="D12" s="32" t="s">
@@ -980,7 +1020,7 @@
       <c r="G12" s="4">
         <v>4</v>
       </c>
-      <c r="H12" s="53">
+      <c r="H12" s="52">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
@@ -992,7 +1032,7 @@
       <c r="B13" s="6">
         <v>8</v>
       </c>
-      <c r="C13" s="49" t="s">
+      <c r="C13" s="48" t="s">
         <v>21</v>
       </c>
       <c r="D13" s="28" t="s">
@@ -1007,7 +1047,7 @@
       <c r="G13" s="5">
         <v>3</v>
       </c>
-      <c r="H13" s="53">
+      <c r="H13" s="52">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
@@ -1035,7 +1075,7 @@
       <c r="G14" s="4">
         <v>5</v>
       </c>
-      <c r="H14" s="52">
+      <c r="H14" s="51">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
@@ -1047,7 +1087,7 @@
       <c r="B15" s="6">
         <v>10</v>
       </c>
-      <c r="C15" s="50" t="s">
+      <c r="C15" s="49" t="s">
         <v>23</v>
       </c>
       <c r="D15" s="17" t="s">
@@ -1062,7 +1102,7 @@
       <c r="G15" s="5">
         <v>3</v>
       </c>
-      <c r="H15" s="53">
+      <c r="H15" s="52">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
@@ -1074,7 +1114,7 @@
       <c r="B16" s="6">
         <v>11</v>
       </c>
-      <c r="C16" s="48" t="s">
+      <c r="C16" s="47" t="s">
         <v>24</v>
       </c>
       <c r="D16" s="18" t="s">
@@ -1089,7 +1129,7 @@
       <c r="G16" s="4">
         <v>2</v>
       </c>
-      <c r="H16" s="53">
+      <c r="H16" s="52">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
@@ -1101,7 +1141,7 @@
       <c r="B17" s="6">
         <v>12</v>
       </c>
-      <c r="C17" s="49" t="s">
+      <c r="C17" s="48" t="s">
         <v>25</v>
       </c>
       <c r="D17" s="27" t="s">
@@ -1116,7 +1156,7 @@
       <c r="G17" s="5">
         <v>1</v>
       </c>
-      <c r="H17" s="53">
+      <c r="H17" s="52">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
@@ -1128,7 +1168,7 @@
       <c r="B18" s="6">
         <v>13</v>
       </c>
-      <c r="C18" s="51" t="s">
+      <c r="C18" s="50" t="s">
         <v>27</v>
       </c>
       <c r="D18" s="20" t="s">
@@ -1143,7 +1183,7 @@
       <c r="G18" s="4">
         <v>1</v>
       </c>
-      <c r="H18" s="53">
+      <c r="H18" s="52">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -1170,7 +1210,7 @@
       <c r="G19" s="5">
         <v>3</v>
       </c>
-      <c r="H19" s="52">
+      <c r="H19" s="51">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
@@ -1182,7 +1222,7 @@
       <c r="B20" s="6">
         <v>15</v>
       </c>
-      <c r="C20" s="48" t="s">
+      <c r="C20" s="47" t="s">
         <v>29</v>
       </c>
       <c r="D20" s="18" t="s">
@@ -1197,7 +1237,7 @@
       <c r="G20" s="4">
         <v>2</v>
       </c>
-      <c r="H20" s="53">
+      <c r="H20" s="52">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
@@ -1224,7 +1264,7 @@
       <c r="G21" s="5">
         <v>5</v>
       </c>
-      <c r="H21" s="52">
+      <c r="H21" s="51">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
@@ -1251,7 +1291,7 @@
       <c r="G22" s="4">
         <v>3</v>
       </c>
-      <c r="H22" s="52">
+      <c r="H22" s="51">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
@@ -1263,7 +1303,7 @@
       <c r="B23" s="6">
         <v>18</v>
       </c>
-      <c r="C23" s="49" t="s">
+      <c r="C23" s="48" t="s">
         <v>34</v>
       </c>
       <c r="D23" s="17" t="s">
@@ -1278,7 +1318,7 @@
       <c r="G23" s="5">
         <v>3</v>
       </c>
-      <c r="H23" s="53">
+      <c r="H23" s="52">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
@@ -1290,7 +1330,7 @@
       <c r="B24" s="6">
         <v>19</v>
       </c>
-      <c r="C24" s="48" t="s">
+      <c r="C24" s="47" t="s">
         <v>35</v>
       </c>
       <c r="D24" s="31" t="s">
@@ -1305,7 +1345,7 @@
       <c r="G24" s="4">
         <v>4</v>
       </c>
-      <c r="H24" s="53">
+      <c r="H24" s="52">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
@@ -1317,7 +1357,7 @@
       <c r="B25" s="6">
         <v>20</v>
       </c>
-      <c r="C25" s="49" t="s">
+      <c r="C25" s="48" t="s">
         <v>37</v>
       </c>
       <c r="D25" s="29" t="s">
@@ -1332,7 +1372,7 @@
       <c r="G25" s="5">
         <v>4</v>
       </c>
-      <c r="H25" s="53">
+      <c r="H25" s="52">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
@@ -1344,7 +1384,7 @@
       <c r="B26" s="6">
         <v>21</v>
       </c>
-      <c r="C26" s="48" t="s">
+      <c r="C26" s="47" t="s">
         <v>38</v>
       </c>
       <c r="D26" s="18" t="s">
@@ -1359,7 +1399,7 @@
       <c r="G26" s="4">
         <v>3</v>
       </c>
-      <c r="H26" s="53">
+      <c r="H26" s="52">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
@@ -1371,7 +1411,7 @@
       <c r="B27" s="6">
         <v>22</v>
       </c>
-      <c r="C27" s="49" t="s">
+      <c r="C27" s="48" t="s">
         <v>39</v>
       </c>
       <c r="D27" s="29" t="s">
@@ -1386,7 +1426,7 @@
       <c r="G27" s="5">
         <v>4</v>
       </c>
-      <c r="H27" s="53">
+      <c r="H27" s="52">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
@@ -1413,7 +1453,7 @@
       <c r="G28" s="4">
         <v>5</v>
       </c>
-      <c r="H28" s="52">
+      <c r="H28" s="51">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
@@ -1425,7 +1465,7 @@
       <c r="B29" s="6">
         <v>24</v>
       </c>
-      <c r="C29" s="49" t="s">
+      <c r="C29" s="48" t="s">
         <v>41</v>
       </c>
       <c r="D29" s="21" t="s">
@@ -1440,7 +1480,7 @@
       <c r="G29" s="5">
         <v>1</v>
       </c>
-      <c r="H29" s="53">
+      <c r="H29" s="52">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -1452,7 +1492,7 @@
       <c r="B30" s="6">
         <v>25</v>
       </c>
-      <c r="C30" s="48" t="s">
+      <c r="C30" s="47" t="s">
         <v>43</v>
       </c>
       <c r="D30" s="20" t="s">
@@ -1467,7 +1507,7 @@
       <c r="G30" s="4">
         <v>1</v>
       </c>
-      <c r="H30" s="53">
+      <c r="H30" s="52">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -1479,7 +1519,7 @@
       <c r="B31" s="6">
         <v>26</v>
       </c>
-      <c r="C31" s="50" t="s">
+      <c r="C31" s="49" t="s">
         <v>44</v>
       </c>
       <c r="D31" s="17" t="s">
@@ -1494,7 +1534,7 @@
       <c r="G31" s="5">
         <v>3</v>
       </c>
-      <c r="H31" s="53">
+      <c r="H31" s="52">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
@@ -1521,7 +1561,7 @@
       <c r="G32" s="4">
         <v>3</v>
       </c>
-      <c r="H32" s="52">
+      <c r="H32" s="51">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
@@ -1533,7 +1573,7 @@
       <c r="B33" s="6">
         <v>28</v>
       </c>
-      <c r="C33" s="49" t="s">
+      <c r="C33" s="48" t="s">
         <v>49</v>
       </c>
       <c r="D33" s="17" t="s">
@@ -1548,7 +1588,7 @@
       <c r="G33" s="5">
         <v>3</v>
       </c>
-      <c r="H33" s="53">
+      <c r="H33" s="52">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
@@ -1560,7 +1600,7 @@
       <c r="B34" s="6">
         <v>29</v>
       </c>
-      <c r="C34" s="48" t="s">
+      <c r="C34" s="47" t="s">
         <v>50</v>
       </c>
       <c r="D34" s="18" t="s">
@@ -1575,7 +1615,7 @@
       <c r="G34" s="4">
         <v>3</v>
       </c>
-      <c r="H34" s="53">
+      <c r="H34" s="52">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
@@ -1587,7 +1627,7 @@
       <c r="B35" s="6">
         <v>30</v>
       </c>
-      <c r="C35" s="48" t="s">
+      <c r="C35" s="47" t="s">
         <v>51</v>
       </c>
       <c r="D35" s="29" t="s">
@@ -1602,7 +1642,7 @@
       <c r="G35" s="5">
         <v>4</v>
       </c>
-      <c r="H35" s="53">
+      <c r="H35" s="52">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
@@ -1614,7 +1654,7 @@
       <c r="B36" s="6">
         <v>31</v>
       </c>
-      <c r="C36" s="45" t="s">
+      <c r="C36" s="53" t="s">
         <v>52</v>
       </c>
       <c r="D36" s="30" t="s">
@@ -1629,7 +1669,7 @@
       <c r="G36" s="4">
         <v>5</v>
       </c>
-      <c r="H36" s="52">
+      <c r="H36" s="54">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -1641,7 +1681,7 @@
       <c r="B37" s="6">
         <v>32</v>
       </c>
-      <c r="C37" s="46" t="s">
+      <c r="C37" s="45" t="s">
         <v>53</v>
       </c>
       <c r="D37" s="17" t="s">
@@ -1656,7 +1696,7 @@
       <c r="G37" s="5">
         <v>4</v>
       </c>
-      <c r="H37" s="52">
+      <c r="H37" s="51">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
@@ -1683,7 +1723,7 @@
       <c r="G38" s="4">
         <v>2</v>
       </c>
-      <c r="H38" s="52">
+      <c r="H38" s="51">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -1695,7 +1735,7 @@
       <c r="B39" s="7">
         <v>34</v>
       </c>
-      <c r="C39" s="50" t="s">
+      <c r="C39" s="49" t="s">
         <v>55</v>
       </c>
       <c r="D39" s="17" t="s">
@@ -1710,7 +1750,7 @@
       <c r="G39" s="5">
         <v>1</v>
       </c>
-      <c r="H39" s="53">
+      <c r="H39" s="52">
         <f>E39*G39</f>
         <v>3</v>
       </c>

</xml_diff>